<commit_message>
Add Predict Droughts results
Wires up the last paper dataset (Kaggle cdminix/us-drought-meteorological-data,
train_timeseries.csv), forward/backward-filling the weekly-only drought score
per county to recover the paper's full 19,300,680-row count. n/k match the
paper's Table 2 exactly for all four features; LightGBM relative accuracy is
in the same ballpark but not an exact match, likely because the paper doesn't
specify how it handles the missing score values.

Raw data (drought.zip and its extracted CSVs) stays out of git per .gitignore;
README documents the Kaggle download.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/boston_531.xlsx
+++ b/boston_531.xlsx
@@ -480,19 +480,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.001313</v>
+        <v>0.001494</v>
       </c>
       <c r="E2" t="n">
         <v>0.9991010299999999</v>
       </c>
       <c r="F2" t="n">
-        <v>0.004118</v>
+        <v>0.004248</v>
       </c>
       <c r="G2" t="n">
         <v>0.892628772</v>
       </c>
       <c r="H2" t="n">
-        <v>0.000162</v>
+        <v>0.000161</v>
       </c>
       <c r="I2" t="n">
         <v>2889.6</v>
@@ -515,19 +515,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.001211</v>
+        <v>0.001242</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.003069</v>
+        <v>0.002341</v>
       </c>
       <c r="G3" t="n">
         <v>0.788635365</v>
       </c>
       <c r="H3" t="n">
-        <v>0.000264</v>
+        <v>0.000265</v>
       </c>
       <c r="I3" t="n">
         <v>2497.9</v>
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.002912</v>
+        <v>0.002877</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004132</v>
+        <v>0.004869</v>
       </c>
       <c r="G4" t="n">
         <v>0.732018476</v>
       </c>
       <c r="H4" t="n">
-        <v>0.000397</v>
+        <v>0.000403</v>
       </c>
       <c r="I4" t="n">
         <v>2283.7</v>

</xml_diff>

<commit_message>
Add synthetic_continuous dataset and refresh Table 2 reproduction
Adds a synthetic dataset (1M rows, 3 categorical features with 10/100/1000
categories, continuous duplicate-free target) to isolate how our_solution's
coordinate-compression trick performs with no target-value duplication to
exploit, the opposite extreme from every real dataset in the registry.
Re-ran the full suite to refresh all result tables accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/boston_531.xlsx
+++ b/boston_531.xlsx
@@ -480,19 +480,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.001494</v>
+        <v>0.001296</v>
       </c>
       <c r="E2" t="n">
         <v>0.9991010299999999</v>
       </c>
       <c r="F2" t="n">
-        <v>0.004248</v>
+        <v>0.005355</v>
       </c>
       <c r="G2" t="n">
         <v>0.892628772</v>
       </c>
       <c r="H2" t="n">
-        <v>0.000161</v>
+        <v>0.000153</v>
       </c>
       <c r="I2" t="n">
         <v>2889.6</v>
@@ -515,19 +515,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.001242</v>
+        <v>0.001182</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>0.002341</v>
+        <v>0.002758</v>
       </c>
       <c r="G3" t="n">
         <v>0.788635365</v>
       </c>
       <c r="H3" t="n">
-        <v>0.000265</v>
+        <v>0.000262</v>
       </c>
       <c r="I3" t="n">
         <v>2497.9</v>
@@ -550,19 +550,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.002877</v>
+        <v>0.002851</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004869</v>
+        <v>0.005307</v>
       </c>
       <c r="G4" t="n">
         <v>0.732018476</v>
       </c>
       <c r="H4" t="n">
-        <v>0.000403</v>
+        <v>0.000395</v>
       </c>
       <c r="I4" t="n">
         <v>2283.7</v>

</xml_diff>